<commit_message>
feat: complete production-ready ARTIX problem collector release
</commit_message>
<xml_diff>
--- a/data/problems.xlsx
+++ b/data/problems.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="41">
   <si>
     <t>ID</t>
   </si>
@@ -116,6 +116,24 @@
   </si>
   <si>
     <t>Salem</t>
+  </si>
+  <si>
+    <t>10:33 PM</t>
+  </si>
+  <si>
+    <t>hi guys naanthaan ungal deva</t>
+  </si>
+  <si>
+    <t>10:34 PM</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>my clg canteen is very bad condition</t>
+  </si>
+  <si>
+    <t>cuddalore</t>
   </si>
 </sst>
 </file>
@@ -550,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -736,6 +754,64 @@
         <v>16</v>
       </c>
     </row>
+    <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>